<commit_message>
added operator and prototypical site number in metadata, update columns in Facility tab
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P1_1stage_noflare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P1_1stage_noflare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wmollel\Documents\MEET2\input\Studies\C3\C3_Prototypical_Sites\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES_development\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B29EE81-B6E6-4456-8050-D117F09441A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2717757B-5F79-4F36-9CE7-2F8719BBCF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="925" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="925" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -1053,7 +1053,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1916,19 +1916,19 @@
         <v>0.14960999999999999</v>
       </c>
       <c r="X2" s="25">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="Y2" s="25">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="Z2" s="25">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="AA2" s="33">
         <v>3000</v>
       </c>
       <c r="AB2" s="33">
-        <v>10000</v>
+        <v>6000</v>
       </c>
       <c r="AC2" s="33">
         <v>5000</v>
@@ -2014,19 +2014,19 @@
         <v>0.14960999999999999</v>
       </c>
       <c r="X3" s="25">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="Y3" s="25">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="Z3" s="25">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="AA3" s="33">
         <v>3000</v>
       </c>
       <c r="AB3" s="33">
-        <v>10000</v>
+        <v>6000</v>
       </c>
       <c r="AC3" s="33">
         <v>5000</v>

</xml_diff>